<commit_message>
Direct Write Excel for QC-10 Day 5
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-10.xlsx
+++ b/FM-MN-07_QC-10.xlsx
@@ -330,7 +330,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
@@ -429,6 +429,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1739,7 +1742,11 @@
       <c r="D6" s="24" t="n"/>
       <c r="E6" s="24" t="n"/>
       <c r="F6" s="24" t="n"/>
-      <c r="G6" s="24" t="n"/>
+      <c r="G6" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="H6" s="24" t="n"/>
       <c r="I6" s="24" t="n"/>
       <c r="J6" s="24" t="n"/>
@@ -1780,7 +1787,11 @@
       <c r="D7" s="24" t="n"/>
       <c r="E7" s="24" t="n"/>
       <c r="F7" s="24" t="n"/>
-      <c r="G7" s="24" t="n"/>
+      <c r="G7" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H7" s="24" t="n"/>
       <c r="I7" s="24" t="n"/>
       <c r="J7" s="24" t="n"/>
@@ -1821,7 +1832,11 @@
       <c r="D8" s="24" t="n"/>
       <c r="E8" s="24" t="n"/>
       <c r="F8" s="24" t="n"/>
-      <c r="G8" s="24" t="n"/>
+      <c r="G8" s="24" t="inlineStr">
+        <is>
+          <t>⨂</t>
+        </is>
+      </c>
       <c r="H8" s="24" t="n"/>
       <c r="I8" s="24" t="n"/>
       <c r="J8" s="24" t="n"/>
@@ -1862,7 +1877,11 @@
       <c r="D9" s="24" t="n"/>
       <c r="E9" s="24" t="n"/>
       <c r="F9" s="24" t="n"/>
-      <c r="G9" s="24" t="n"/>
+      <c r="G9" s="24" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H9" s="24" t="n"/>
       <c r="I9" s="24" t="n"/>
       <c r="J9" s="24" t="n"/>
@@ -1897,7 +1916,11 @@
       <c r="D10" s="38" t="n"/>
       <c r="E10" s="38" t="n"/>
       <c r="F10" s="38" t="n"/>
-      <c r="G10" s="38" t="n"/>
+      <c r="G10" s="40" t="inlineStr">
+        <is>
+          <t>เค</t>
+        </is>
+      </c>
       <c r="H10" s="38" t="n"/>
       <c r="I10" s="38" t="n"/>
       <c r="J10" s="38" t="n"/>
@@ -2078,8 +2101,8 @@
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="AA10:AA11"/>
     <mergeCell ref="E10:E11"/>
+    <mergeCell ref="V10:V11"/>
     <mergeCell ref="Z12:Z13"/>
-    <mergeCell ref="V10:V11"/>
     <mergeCell ref="G10:G11"/>
     <mergeCell ref="M10:M11"/>
     <mergeCell ref="AB12:AB13"/>

</xml_diff>

<commit_message>
Reset Excel Table for QC-10
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-10.xlsx
+++ b/FM-MN-07_QC-10.xlsx
@@ -1741,41 +1741,37 @@
           <t>ตรวจดูสภาพของไมโครพร้อมใช้งานหรือไม่</t>
         </is>
       </c>
-      <c r="C6" s="24" t="n"/>
-      <c r="D6" s="24" t="n"/>
-      <c r="E6" s="24" t="n"/>
-      <c r="F6" s="24" t="n"/>
-      <c r="G6" s="24" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="H6" s="24" t="n"/>
-      <c r="I6" s="24" t="n"/>
-      <c r="J6" s="24" t="n"/>
-      <c r="K6" s="24" t="n"/>
-      <c r="L6" s="24" t="n"/>
-      <c r="M6" s="24" t="n"/>
-      <c r="N6" s="24" t="n"/>
-      <c r="O6" s="24" t="n"/>
-      <c r="P6" s="24" t="n"/>
-      <c r="Q6" s="24" t="n"/>
-      <c r="R6" s="24" t="n"/>
-      <c r="S6" s="24" t="n"/>
-      <c r="T6" s="24" t="n"/>
-      <c r="U6" s="24" t="n"/>
-      <c r="V6" s="24" t="n"/>
-      <c r="W6" s="24" t="n"/>
-      <c r="X6" s="24" t="n"/>
-      <c r="Y6" s="24" t="n"/>
-      <c r="Z6" s="24" t="n"/>
-      <c r="AA6" s="24" t="n"/>
-      <c r="AB6" s="24" t="n"/>
-      <c r="AC6" s="24" t="n"/>
-      <c r="AD6" s="24" t="n"/>
-      <c r="AE6" s="24" t="n"/>
-      <c r="AF6" s="24" t="n"/>
-      <c r="AG6" s="24" t="n"/>
+      <c r="C6" s="24" t="inlineStr"/>
+      <c r="D6" s="24" t="inlineStr"/>
+      <c r="E6" s="24" t="inlineStr"/>
+      <c r="F6" s="24" t="inlineStr"/>
+      <c r="G6" s="24" t="inlineStr"/>
+      <c r="H6" s="24" t="inlineStr"/>
+      <c r="I6" s="24" t="inlineStr"/>
+      <c r="J6" s="24" t="inlineStr"/>
+      <c r="K6" s="24" t="inlineStr"/>
+      <c r="L6" s="24" t="inlineStr"/>
+      <c r="M6" s="24" t="inlineStr"/>
+      <c r="N6" s="24" t="inlineStr"/>
+      <c r="O6" s="24" t="inlineStr"/>
+      <c r="P6" s="24" t="inlineStr"/>
+      <c r="Q6" s="24" t="inlineStr"/>
+      <c r="R6" s="24" t="inlineStr"/>
+      <c r="S6" s="24" t="inlineStr"/>
+      <c r="T6" s="24" t="inlineStr"/>
+      <c r="U6" s="24" t="inlineStr"/>
+      <c r="V6" s="24" t="inlineStr"/>
+      <c r="W6" s="24" t="inlineStr"/>
+      <c r="X6" s="24" t="inlineStr"/>
+      <c r="Y6" s="24" t="inlineStr"/>
+      <c r="Z6" s="24" t="inlineStr"/>
+      <c r="AA6" s="24" t="inlineStr"/>
+      <c r="AB6" s="24" t="inlineStr"/>
+      <c r="AC6" s="24" t="inlineStr"/>
+      <c r="AD6" s="24" t="inlineStr"/>
+      <c r="AE6" s="24" t="inlineStr"/>
+      <c r="AF6" s="24" t="inlineStr"/>
+      <c r="AG6" s="24" t="inlineStr"/>
     </row>
     <row r="7" ht="15.75" customFormat="1" customHeight="1" s="9">
       <c r="A7" s="12" t="n">
@@ -1786,41 +1782,37 @@
           <t>ตรวจดู BATTERRY อ่อนหรือไม่</t>
         </is>
       </c>
-      <c r="C7" s="24" t="n"/>
-      <c r="D7" s="24" t="n"/>
-      <c r="E7" s="24" t="n"/>
-      <c r="F7" s="24" t="n"/>
-      <c r="G7" s="24" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H7" s="24" t="n"/>
-      <c r="I7" s="24" t="n"/>
-      <c r="J7" s="24" t="n"/>
-      <c r="K7" s="24" t="n"/>
-      <c r="L7" s="24" t="n"/>
-      <c r="M7" s="24" t="n"/>
-      <c r="N7" s="24" t="n"/>
-      <c r="O7" s="24" t="n"/>
-      <c r="P7" s="24" t="n"/>
-      <c r="Q7" s="24" t="n"/>
-      <c r="R7" s="24" t="n"/>
-      <c r="S7" s="24" t="n"/>
-      <c r="T7" s="24" t="n"/>
-      <c r="U7" s="24" t="n"/>
-      <c r="V7" s="24" t="n"/>
-      <c r="W7" s="24" t="n"/>
-      <c r="X7" s="24" t="n"/>
-      <c r="Y7" s="24" t="n"/>
-      <c r="Z7" s="24" t="n"/>
-      <c r="AA7" s="24" t="n"/>
-      <c r="AB7" s="24" t="n"/>
-      <c r="AC7" s="24" t="n"/>
-      <c r="AD7" s="24" t="n"/>
-      <c r="AE7" s="24" t="n"/>
-      <c r="AF7" s="24" t="n"/>
-      <c r="AG7" s="24" t="n"/>
+      <c r="C7" s="24" t="inlineStr"/>
+      <c r="D7" s="24" t="inlineStr"/>
+      <c r="E7" s="24" t="inlineStr"/>
+      <c r="F7" s="24" t="inlineStr"/>
+      <c r="G7" s="24" t="inlineStr"/>
+      <c r="H7" s="24" t="inlineStr"/>
+      <c r="I7" s="24" t="inlineStr"/>
+      <c r="J7" s="24" t="inlineStr"/>
+      <c r="K7" s="24" t="inlineStr"/>
+      <c r="L7" s="24" t="inlineStr"/>
+      <c r="M7" s="24" t="inlineStr"/>
+      <c r="N7" s="24" t="inlineStr"/>
+      <c r="O7" s="24" t="inlineStr"/>
+      <c r="P7" s="24" t="inlineStr"/>
+      <c r="Q7" s="24" t="inlineStr"/>
+      <c r="R7" s="24" t="inlineStr"/>
+      <c r="S7" s="24" t="inlineStr"/>
+      <c r="T7" s="24" t="inlineStr"/>
+      <c r="U7" s="24" t="inlineStr"/>
+      <c r="V7" s="24" t="inlineStr"/>
+      <c r="W7" s="24" t="inlineStr"/>
+      <c r="X7" s="24" t="inlineStr"/>
+      <c r="Y7" s="24" t="inlineStr"/>
+      <c r="Z7" s="24" t="inlineStr"/>
+      <c r="AA7" s="24" t="inlineStr"/>
+      <c r="AB7" s="24" t="inlineStr"/>
+      <c r="AC7" s="24" t="inlineStr"/>
+      <c r="AD7" s="24" t="inlineStr"/>
+      <c r="AE7" s="24" t="inlineStr"/>
+      <c r="AF7" s="24" t="inlineStr"/>
+      <c r="AG7" s="24" t="inlineStr"/>
     </row>
     <row r="8" ht="15.75" customFormat="1" customHeight="1" s="9">
       <c r="A8" s="12" t="n">
@@ -1831,41 +1823,37 @@
           <t>ตรวจสอบการสไลด์ต้องไม่ติดขัด</t>
         </is>
       </c>
-      <c r="C8" s="24" t="n"/>
-      <c r="D8" s="24" t="n"/>
-      <c r="E8" s="24" t="n"/>
-      <c r="F8" s="24" t="n"/>
-      <c r="G8" s="24" t="inlineStr">
-        <is>
-          <t>⨂</t>
-        </is>
-      </c>
-      <c r="H8" s="24" t="n"/>
-      <c r="I8" s="24" t="n"/>
-      <c r="J8" s="24" t="n"/>
-      <c r="K8" s="24" t="n"/>
-      <c r="L8" s="24" t="n"/>
-      <c r="M8" s="24" t="n"/>
-      <c r="N8" s="24" t="n"/>
-      <c r="O8" s="24" t="n"/>
-      <c r="P8" s="24" t="n"/>
-      <c r="Q8" s="24" t="n"/>
-      <c r="R8" s="24" t="n"/>
-      <c r="S8" s="24" t="n"/>
-      <c r="T8" s="24" t="n"/>
-      <c r="U8" s="24" t="n"/>
-      <c r="V8" s="24" t="n"/>
-      <c r="W8" s="24" t="n"/>
-      <c r="X8" s="24" t="n"/>
-      <c r="Y8" s="24" t="n"/>
-      <c r="Z8" s="24" t="n"/>
-      <c r="AA8" s="24" t="n"/>
-      <c r="AB8" s="24" t="n"/>
-      <c r="AC8" s="24" t="n"/>
-      <c r="AD8" s="24" t="n"/>
-      <c r="AE8" s="24" t="n"/>
-      <c r="AF8" s="24" t="n"/>
-      <c r="AG8" s="24" t="n"/>
+      <c r="C8" s="24" t="inlineStr"/>
+      <c r="D8" s="24" t="inlineStr"/>
+      <c r="E8" s="24" t="inlineStr"/>
+      <c r="F8" s="24" t="inlineStr"/>
+      <c r="G8" s="24" t="inlineStr"/>
+      <c r="H8" s="24" t="inlineStr"/>
+      <c r="I8" s="24" t="inlineStr"/>
+      <c r="J8" s="24" t="inlineStr"/>
+      <c r="K8" s="24" t="inlineStr"/>
+      <c r="L8" s="24" t="inlineStr"/>
+      <c r="M8" s="24" t="inlineStr"/>
+      <c r="N8" s="24" t="inlineStr"/>
+      <c r="O8" s="24" t="inlineStr"/>
+      <c r="P8" s="24" t="inlineStr"/>
+      <c r="Q8" s="24" t="inlineStr"/>
+      <c r="R8" s="24" t="inlineStr"/>
+      <c r="S8" s="24" t="inlineStr"/>
+      <c r="T8" s="24" t="inlineStr"/>
+      <c r="U8" s="24" t="inlineStr"/>
+      <c r="V8" s="24" t="inlineStr"/>
+      <c r="W8" s="24" t="inlineStr"/>
+      <c r="X8" s="24" t="inlineStr"/>
+      <c r="Y8" s="24" t="inlineStr"/>
+      <c r="Z8" s="24" t="inlineStr"/>
+      <c r="AA8" s="24" t="inlineStr"/>
+      <c r="AB8" s="24" t="inlineStr"/>
+      <c r="AC8" s="24" t="inlineStr"/>
+      <c r="AD8" s="24" t="inlineStr"/>
+      <c r="AE8" s="24" t="inlineStr"/>
+      <c r="AF8" s="24" t="inlineStr"/>
+      <c r="AG8" s="24" t="inlineStr"/>
     </row>
     <row r="9" ht="15.75" customFormat="1" customHeight="1" s="9">
       <c r="A9" s="12" t="n">
@@ -1876,80 +1864,72 @@
           <t>หลังเลิกงานต้องปิดสวิตส์ทุกครั้ง</t>
         </is>
       </c>
-      <c r="C9" s="24" t="n"/>
-      <c r="D9" s="24" t="n"/>
-      <c r="E9" s="24" t="n"/>
-      <c r="F9" s="24" t="n"/>
-      <c r="G9" s="24" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H9" s="24" t="n"/>
-      <c r="I9" s="24" t="n"/>
-      <c r="J9" s="24" t="n"/>
-      <c r="K9" s="24" t="n"/>
-      <c r="L9" s="24" t="n"/>
-      <c r="M9" s="24" t="n"/>
-      <c r="N9" s="24" t="n"/>
-      <c r="O9" s="24" t="n"/>
-      <c r="P9" s="24" t="n"/>
-      <c r="Q9" s="24" t="n"/>
-      <c r="R9" s="24" t="n"/>
-      <c r="S9" s="24" t="n"/>
-      <c r="T9" s="24" t="n"/>
-      <c r="U9" s="24" t="n"/>
-      <c r="V9" s="24" t="n"/>
-      <c r="W9" s="24" t="n"/>
-      <c r="X9" s="24" t="n"/>
-      <c r="Y9" s="24" t="n"/>
-      <c r="Z9" s="24" t="n"/>
-      <c r="AA9" s="24" t="n"/>
-      <c r="AB9" s="24" t="n"/>
-      <c r="AC9" s="24" t="n"/>
-      <c r="AD9" s="24" t="n"/>
-      <c r="AE9" s="24" t="n"/>
-      <c r="AF9" s="24" t="n"/>
-      <c r="AG9" s="24" t="n"/>
+      <c r="C9" s="24" t="inlineStr"/>
+      <c r="D9" s="24" t="inlineStr"/>
+      <c r="E9" s="24" t="inlineStr"/>
+      <c r="F9" s="24" t="inlineStr"/>
+      <c r="G9" s="24" t="inlineStr"/>
+      <c r="H9" s="24" t="inlineStr"/>
+      <c r="I9" s="24" t="inlineStr"/>
+      <c r="J9" s="24" t="inlineStr"/>
+      <c r="K9" s="24" t="inlineStr"/>
+      <c r="L9" s="24" t="inlineStr"/>
+      <c r="M9" s="24" t="inlineStr"/>
+      <c r="N9" s="24" t="inlineStr"/>
+      <c r="O9" s="24" t="inlineStr"/>
+      <c r="P9" s="24" t="inlineStr"/>
+      <c r="Q9" s="24" t="inlineStr"/>
+      <c r="R9" s="24" t="inlineStr"/>
+      <c r="S9" s="24" t="inlineStr"/>
+      <c r="T9" s="24" t="inlineStr"/>
+      <c r="U9" s="24" t="inlineStr"/>
+      <c r="V9" s="24" t="inlineStr"/>
+      <c r="W9" s="24" t="inlineStr"/>
+      <c r="X9" s="24" t="inlineStr"/>
+      <c r="Y9" s="24" t="inlineStr"/>
+      <c r="Z9" s="24" t="inlineStr"/>
+      <c r="AA9" s="24" t="inlineStr"/>
+      <c r="AB9" s="24" t="inlineStr"/>
+      <c r="AC9" s="24" t="inlineStr"/>
+      <c r="AD9" s="24" t="inlineStr"/>
+      <c r="AE9" s="24" t="inlineStr"/>
+      <c r="AF9" s="24" t="inlineStr"/>
+      <c r="AG9" s="24" t="inlineStr"/>
     </row>
     <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="8" t="n"/>
       <c r="B10" s="7" t="n"/>
-      <c r="C10" s="38" t="n"/>
-      <c r="D10" s="38" t="n"/>
-      <c r="E10" s="38" t="n"/>
-      <c r="F10" s="38" t="n"/>
-      <c r="G10" s="40" t="inlineStr">
-        <is>
-          <t>เค</t>
-        </is>
-      </c>
-      <c r="H10" s="38" t="n"/>
-      <c r="I10" s="38" t="n"/>
-      <c r="J10" s="38" t="n"/>
-      <c r="K10" s="38" t="n"/>
-      <c r="L10" s="38" t="n"/>
-      <c r="M10" s="38" t="n"/>
-      <c r="N10" s="38" t="n"/>
-      <c r="O10" s="38" t="n"/>
-      <c r="P10" s="38" t="n"/>
-      <c r="Q10" s="38" t="n"/>
-      <c r="R10" s="38" t="n"/>
-      <c r="S10" s="38" t="n"/>
-      <c r="T10" s="38" t="n"/>
-      <c r="U10" s="38" t="n"/>
-      <c r="V10" s="38" t="n"/>
-      <c r="W10" s="38" t="n"/>
-      <c r="X10" s="38" t="n"/>
-      <c r="Y10" s="38" t="n"/>
-      <c r="Z10" s="38" t="n"/>
-      <c r="AA10" s="38" t="n"/>
-      <c r="AB10" s="38" t="n"/>
-      <c r="AC10" s="38" t="n"/>
-      <c r="AD10" s="38" t="n"/>
-      <c r="AE10" s="38" t="n"/>
-      <c r="AF10" s="38" t="n"/>
-      <c r="AG10" s="38" t="n"/>
+      <c r="C10" s="38" t="inlineStr"/>
+      <c r="D10" s="38" t="inlineStr"/>
+      <c r="E10" s="38" t="inlineStr"/>
+      <c r="F10" s="38" t="inlineStr"/>
+      <c r="G10" s="40" t="inlineStr"/>
+      <c r="H10" s="38" t="inlineStr"/>
+      <c r="I10" s="38" t="inlineStr"/>
+      <c r="J10" s="38" t="inlineStr"/>
+      <c r="K10" s="38" t="inlineStr"/>
+      <c r="L10" s="38" t="inlineStr"/>
+      <c r="M10" s="38" t="inlineStr"/>
+      <c r="N10" s="38" t="inlineStr"/>
+      <c r="O10" s="38" t="inlineStr"/>
+      <c r="P10" s="38" t="inlineStr"/>
+      <c r="Q10" s="38" t="inlineStr"/>
+      <c r="R10" s="38" t="inlineStr"/>
+      <c r="S10" s="38" t="inlineStr"/>
+      <c r="T10" s="38" t="inlineStr"/>
+      <c r="U10" s="38" t="inlineStr"/>
+      <c r="V10" s="38" t="inlineStr"/>
+      <c r="W10" s="38" t="inlineStr"/>
+      <c r="X10" s="38" t="inlineStr"/>
+      <c r="Y10" s="38" t="inlineStr"/>
+      <c r="Z10" s="38" t="inlineStr"/>
+      <c r="AA10" s="38" t="inlineStr"/>
+      <c r="AB10" s="38" t="inlineStr"/>
+      <c r="AC10" s="38" t="inlineStr"/>
+      <c r="AD10" s="38" t="inlineStr"/>
+      <c r="AE10" s="38" t="inlineStr"/>
+      <c r="AF10" s="38" t="inlineStr"/>
+      <c r="AG10" s="38" t="inlineStr"/>
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="B11" s="6" t="n"/>
@@ -1987,41 +1967,37 @@
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="B12" s="6" t="n"/>
-      <c r="C12" s="21" t="n"/>
-      <c r="D12" s="21" t="n"/>
-      <c r="E12" s="21" t="n"/>
-      <c r="F12" s="21" t="n"/>
-      <c r="G12" s="41" t="inlineStr">
-        <is>
-          <t>พลวัฒน์</t>
-        </is>
-      </c>
-      <c r="H12" s="21" t="n"/>
-      <c r="I12" s="21" t="n"/>
-      <c r="J12" s="21" t="n"/>
-      <c r="K12" s="21" t="n"/>
-      <c r="L12" s="21" t="n"/>
-      <c r="M12" s="21" t="n"/>
-      <c r="N12" s="21" t="n"/>
-      <c r="O12" s="21" t="n"/>
-      <c r="P12" s="21" t="n"/>
-      <c r="Q12" s="21" t="n"/>
-      <c r="R12" s="21" t="n"/>
-      <c r="S12" s="21" t="n"/>
-      <c r="T12" s="21" t="n"/>
-      <c r="U12" s="21" t="n"/>
-      <c r="V12" s="21" t="n"/>
-      <c r="W12" s="21" t="n"/>
-      <c r="X12" s="21" t="n"/>
-      <c r="Y12" s="21" t="n"/>
-      <c r="Z12" s="21" t="n"/>
-      <c r="AA12" s="21" t="n"/>
-      <c r="AB12" s="21" t="n"/>
-      <c r="AC12" s="21" t="n"/>
-      <c r="AD12" s="21" t="n"/>
-      <c r="AE12" s="21" t="n"/>
-      <c r="AF12" s="21" t="n"/>
-      <c r="AG12" s="21" t="n"/>
+      <c r="C12" s="21" t="inlineStr"/>
+      <c r="D12" s="21" t="inlineStr"/>
+      <c r="E12" s="21" t="inlineStr"/>
+      <c r="F12" s="21" t="inlineStr"/>
+      <c r="G12" s="41" t="inlineStr"/>
+      <c r="H12" s="21" t="inlineStr"/>
+      <c r="I12" s="21" t="inlineStr"/>
+      <c r="J12" s="21" t="inlineStr"/>
+      <c r="K12" s="21" t="inlineStr"/>
+      <c r="L12" s="21" t="inlineStr"/>
+      <c r="M12" s="21" t="inlineStr"/>
+      <c r="N12" s="21" t="inlineStr"/>
+      <c r="O12" s="21" t="inlineStr"/>
+      <c r="P12" s="21" t="inlineStr"/>
+      <c r="Q12" s="21" t="inlineStr"/>
+      <c r="R12" s="21" t="inlineStr"/>
+      <c r="S12" s="21" t="inlineStr"/>
+      <c r="T12" s="21" t="inlineStr"/>
+      <c r="U12" s="21" t="inlineStr"/>
+      <c r="V12" s="21" t="inlineStr"/>
+      <c r="W12" s="21" t="inlineStr"/>
+      <c r="X12" s="21" t="inlineStr"/>
+      <c r="Y12" s="21" t="inlineStr"/>
+      <c r="Z12" s="21" t="inlineStr"/>
+      <c r="AA12" s="21" t="inlineStr"/>
+      <c r="AB12" s="21" t="inlineStr"/>
+      <c r="AC12" s="21" t="inlineStr"/>
+      <c r="AD12" s="21" t="inlineStr"/>
+      <c r="AE12" s="21" t="inlineStr"/>
+      <c r="AF12" s="21" t="inlineStr"/>
+      <c r="AG12" s="21" t="inlineStr"/>
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="B13" s="6" t="n"/>
@@ -2065,7 +2041,7 @@
       </c>
     </row>
     <row r="15" ht="185.25" customHeight="1">
-      <c r="B15" s="32" t="n"/>
+      <c r="B15" s="32" t="inlineStr"/>
     </row>
     <row r="16" ht="23.25" customHeight="1"/>
     <row r="17" ht="21" customHeight="1">
@@ -2107,9 +2083,9 @@
     <mergeCell ref="N12:N13"/>
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="AA10:AA11"/>
-    <mergeCell ref="V10:V11"/>
     <mergeCell ref="E10:E11"/>
     <mergeCell ref="Z12:Z13"/>
+    <mergeCell ref="V10:V11"/>
     <mergeCell ref="G10:G11"/>
     <mergeCell ref="M10:M11"/>
     <mergeCell ref="AB12:AB13"/>

</xml_diff>

<commit_message>
Direct Write Excel for QC-10 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-10.xlsx
+++ b/FM-MN-07_QC-10.xlsx
@@ -1746,7 +1746,11 @@
       <c r="E6" s="24" t="inlineStr"/>
       <c r="F6" s="24" t="inlineStr"/>
       <c r="G6" s="24" t="inlineStr"/>
-      <c r="H6" s="24" t="inlineStr"/>
+      <c r="H6" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I6" s="24" t="inlineStr"/>
       <c r="J6" s="24" t="inlineStr"/>
       <c r="K6" s="24" t="inlineStr"/>
@@ -1787,7 +1791,11 @@
       <c r="E7" s="24" t="inlineStr"/>
       <c r="F7" s="24" t="inlineStr"/>
       <c r="G7" s="24" t="inlineStr"/>
-      <c r="H7" s="24" t="inlineStr"/>
+      <c r="H7" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I7" s="24" t="inlineStr"/>
       <c r="J7" s="24" t="inlineStr"/>
       <c r="K7" s="24" t="inlineStr"/>
@@ -1828,7 +1836,11 @@
       <c r="E8" s="24" t="inlineStr"/>
       <c r="F8" s="24" t="inlineStr"/>
       <c r="G8" s="24" t="inlineStr"/>
-      <c r="H8" s="24" t="inlineStr"/>
+      <c r="H8" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I8" s="24" t="inlineStr"/>
       <c r="J8" s="24" t="inlineStr"/>
       <c r="K8" s="24" t="inlineStr"/>
@@ -1869,7 +1881,11 @@
       <c r="E9" s="24" t="inlineStr"/>
       <c r="F9" s="24" t="inlineStr"/>
       <c r="G9" s="24" t="inlineStr"/>
-      <c r="H9" s="24" t="inlineStr"/>
+      <c r="H9" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I9" s="24" t="inlineStr"/>
       <c r="J9" s="24" t="inlineStr"/>
       <c r="K9" s="24" t="inlineStr"/>
@@ -1904,7 +1920,11 @@
       <c r="E10" s="38" t="inlineStr"/>
       <c r="F10" s="38" t="inlineStr"/>
       <c r="G10" s="40" t="inlineStr"/>
-      <c r="H10" s="38" t="inlineStr"/>
+      <c r="H10" s="40" t="inlineStr">
+        <is>
+          <t>สัมพันธ์ รักวิถี</t>
+        </is>
+      </c>
       <c r="I10" s="38" t="inlineStr"/>
       <c r="J10" s="38" t="inlineStr"/>
       <c r="K10" s="38" t="inlineStr"/>
@@ -2084,8 +2104,8 @@
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="AA10:AA11"/>
     <mergeCell ref="E10:E11"/>
+    <mergeCell ref="V10:V11"/>
     <mergeCell ref="Z12:Z13"/>
-    <mergeCell ref="V10:V11"/>
     <mergeCell ref="G10:G11"/>
     <mergeCell ref="M10:M11"/>
     <mergeCell ref="AB12:AB13"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for QC-10 Day 7
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-10.xlsx
+++ b/FM-MN-07_QC-10.xlsx
@@ -1751,7 +1751,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I6" s="24" t="inlineStr"/>
+      <c r="I6" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J6" s="24" t="inlineStr"/>
       <c r="K6" s="24" t="inlineStr"/>
       <c r="L6" s="24" t="inlineStr"/>
@@ -1796,7 +1800,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I7" s="24" t="inlineStr"/>
+      <c r="I7" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J7" s="24" t="inlineStr"/>
       <c r="K7" s="24" t="inlineStr"/>
       <c r="L7" s="24" t="inlineStr"/>
@@ -1841,7 +1849,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I8" s="24" t="inlineStr"/>
+      <c r="I8" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J8" s="24" t="inlineStr"/>
       <c r="K8" s="24" t="inlineStr"/>
       <c r="L8" s="24" t="inlineStr"/>
@@ -1886,7 +1898,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I9" s="24" t="inlineStr"/>
+      <c r="I9" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J9" s="24" t="inlineStr"/>
       <c r="K9" s="24" t="inlineStr"/>
       <c r="L9" s="24" t="inlineStr"/>
@@ -2107,9 +2123,9 @@
     <mergeCell ref="N12:N13"/>
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="AA10:AA11"/>
-    <mergeCell ref="V10:V11"/>
     <mergeCell ref="E10:E11"/>
     <mergeCell ref="Z12:Z13"/>
+    <mergeCell ref="V10:V11"/>
     <mergeCell ref="G10:G11"/>
     <mergeCell ref="M10:M11"/>
     <mergeCell ref="AB12:AB13"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for QC-10 Day 8
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-10.xlsx
+++ b/FM-MN-07_QC-10.xlsx
@@ -1756,7 +1756,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J6" s="24" t="inlineStr"/>
+      <c r="J6" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K6" s="24" t="inlineStr"/>
       <c r="L6" s="24" t="inlineStr"/>
       <c r="M6" s="24" t="inlineStr"/>
@@ -1805,7 +1809,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J7" s="24" t="inlineStr"/>
+      <c r="J7" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K7" s="24" t="inlineStr"/>
       <c r="L7" s="24" t="inlineStr"/>
       <c r="M7" s="24" t="inlineStr"/>
@@ -1854,7 +1862,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J8" s="24" t="inlineStr"/>
+      <c r="J8" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K8" s="24" t="inlineStr"/>
       <c r="L8" s="24" t="inlineStr"/>
       <c r="M8" s="24" t="inlineStr"/>
@@ -1903,7 +1915,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J9" s="24" t="inlineStr"/>
+      <c r="J9" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K9" s="24" t="inlineStr"/>
       <c r="L9" s="24" t="inlineStr"/>
       <c r="M9" s="24" t="inlineStr"/>
@@ -2124,8 +2140,8 @@
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="AA10:AA11"/>
     <mergeCell ref="E10:E11"/>
+    <mergeCell ref="V10:V11"/>
     <mergeCell ref="Z12:Z13"/>
-    <mergeCell ref="V10:V11"/>
     <mergeCell ref="G10:G11"/>
     <mergeCell ref="M10:M11"/>
     <mergeCell ref="AB12:AB13"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for QC-10 Day 10
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-10.xlsx
+++ b/FM-MN-07_QC-10.xlsx
@@ -1762,7 +1762,11 @@
         </is>
       </c>
       <c r="K6" s="24" t="inlineStr"/>
-      <c r="L6" s="24" t="inlineStr"/>
+      <c r="L6" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M6" s="24" t="inlineStr"/>
       <c r="N6" s="24" t="inlineStr"/>
       <c r="O6" s="24" t="inlineStr"/>
@@ -1815,7 +1819,11 @@
         </is>
       </c>
       <c r="K7" s="24" t="inlineStr"/>
-      <c r="L7" s="24" t="inlineStr"/>
+      <c r="L7" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M7" s="24" t="inlineStr"/>
       <c r="N7" s="24" t="inlineStr"/>
       <c r="O7" s="24" t="inlineStr"/>
@@ -1868,7 +1876,11 @@
         </is>
       </c>
       <c r="K8" s="24" t="inlineStr"/>
-      <c r="L8" s="24" t="inlineStr"/>
+      <c r="L8" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M8" s="24" t="inlineStr"/>
       <c r="N8" s="24" t="inlineStr"/>
       <c r="O8" s="24" t="inlineStr"/>
@@ -1921,7 +1933,11 @@
         </is>
       </c>
       <c r="K9" s="24" t="inlineStr"/>
-      <c r="L9" s="24" t="inlineStr"/>
+      <c r="L9" s="24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M9" s="24" t="inlineStr"/>
       <c r="N9" s="24" t="inlineStr"/>
       <c r="O9" s="24" t="inlineStr"/>
@@ -2139,8 +2155,8 @@
     <mergeCell ref="N12:N13"/>
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="AA10:AA11"/>
+    <mergeCell ref="V10:V11"/>
     <mergeCell ref="E10:E11"/>
-    <mergeCell ref="V10:V11"/>
     <mergeCell ref="Z12:Z13"/>
     <mergeCell ref="G10:G11"/>
     <mergeCell ref="M10:M11"/>

</xml_diff>